<commit_message>
Strip the storage path and author properties from the refinement workbook
RietveldSummary.xlsx carried the personal cloud-storage path it was last saved from,
in xl/workbook.xml, along with a revision pointer, and author, editor and date
properties in docProps/core.xml. None of that is data. Those two parts are rewritten
without it; every other part of the package, the cell values, formulas and chart
included, is byte-identical to the file as received.
</commit_message>
<xml_diff>
--- a/Data/xrd/RietveldSummary.xlsx
+++ b/Data/xrd/RietveldSummary.xlsx
@@ -3,12 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ornl-my.sharepoint.com/personal/6d1_ornl_gov/Documents/Materials_ML/Alicia/CeO2_Nd_XRD/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="122" documentId="8_{E22D68ED-1AB3-A846-B34C-01D3ADE1FEC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7AF2D7E0-A181-4191-9762-E98D6C511CAF}"/>
   <bookViews>
     <workbookView xWindow="10" yWindow="730" windowWidth="19190" windowHeight="11270" xr2:uid="{3DF5CA76-8770-D249-8FF3-BB482DB4554C}"/>
   </bookViews>

</xml_diff>